<commit_message>
Update database structure Excel file and remove temporary file
</commit_message>
<xml_diff>
--- a/data/estructura_bbdd.xlsx
+++ b/data/estructura_bbdd.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomas/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomas/GitHub/ele7/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F3CFB2D-4629-9C4A-9E9A-519AAD634D03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE9419B-ED10-1443-A5A6-339813539765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36000" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36060" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Codificacion_formulario_ELE7" sheetId="4" r:id="rId1"/>
@@ -6028,6 +6028,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:V772"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -6035,7 +6036,7 @@
     <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.5" customWidth="1"/>
-    <col min="5" max="5" width="43.33203125" customWidth="1"/>
+    <col min="5" max="5" width="159.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.33203125" style="38" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="42.33203125" customWidth="1"/>
     <col min="8" max="8" width="19.83203125" customWidth="1"/>
@@ -6340,7 +6341,7 @@
         <v>1518</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>1</v>
       </c>
@@ -6375,7 +6376,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>1</v>
       </c>
@@ -6410,7 +6411,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>1</v>
       </c>
@@ -6445,7 +6446,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>1</v>
       </c>
@@ -6480,7 +6481,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>1</v>
       </c>
@@ -6515,7 +6516,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>1</v>
       </c>
@@ -6550,7 +6551,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4">
         <v>1</v>
       </c>
@@ -6585,7 +6586,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4">
         <v>1</v>
       </c>
@@ -6620,7 +6621,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4">
         <v>1</v>
       </c>
@@ -6655,7 +6656,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4">
         <v>1</v>
       </c>
@@ -6690,7 +6691,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4">
         <v>1</v>
       </c>
@@ -6725,7 +6726,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4">
         <v>1</v>
       </c>
@@ -6760,7 +6761,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4">
         <v>1</v>
       </c>
@@ -6795,7 +6796,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4">
         <v>1</v>
       </c>
@@ -6830,7 +6831,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4">
         <v>1</v>
       </c>
@@ -6865,7 +6866,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4">
         <v>1</v>
       </c>
@@ -6902,7 +6903,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4">
         <v>1</v>
       </c>
@@ -6939,7 +6940,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4">
         <v>1</v>
       </c>
@@ -6976,7 +6977,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4">
         <v>1</v>
       </c>
@@ -7259,7 +7260,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4">
         <v>1</v>
       </c>
@@ -7298,7 +7299,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4">
         <v>1</v>
       </c>
@@ -7337,7 +7338,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4">
         <v>1</v>
       </c>
@@ -7376,7 +7377,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4">
         <v>1</v>
       </c>
@@ -7415,7 +7416,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4">
         <v>1</v>
       </c>
@@ -7454,7 +7455,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4">
         <v>1</v>
       </c>
@@ -7493,7 +7494,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4">
         <v>1</v>
       </c>
@@ -7770,7 +7771,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4">
         <v>1</v>
       </c>
@@ -8500,7 +8501,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:13" ht="49.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="4">
         <v>1</v>
       </c>
@@ -8859,7 +8860,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="76" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:13" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="4">
         <v>1</v>
       </c>
@@ -9179,7 +9180,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="84" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:13" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="4">
         <v>1</v>
       </c>
@@ -9710,7 +9711,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="97" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:13" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" s="4">
         <v>2</v>
       </c>
@@ -10443,7 +10444,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="115" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:13" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" s="4">
         <v>2</v>
       </c>
@@ -11220,7 +11221,7 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="134" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" s="4">
         <v>2</v>
       </c>
@@ -11546,7 +11547,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="142" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:13" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A142" s="4">
         <v>2</v>
       </c>
@@ -11790,7 +11791,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="148" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A148" s="4">
         <v>2</v>
       </c>
@@ -12114,7 +12115,7 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="156" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:13" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A156" s="4">
         <v>2</v>
       </c>
@@ -12354,7 +12355,7 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="162" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:13" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A162" s="4">
         <v>2</v>
       </c>
@@ -12803,7 +12804,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="173" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:13" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A173" s="4">
         <v>2</v>
       </c>
@@ -13170,7 +13171,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="182" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A182" s="4">
         <v>2</v>
       </c>
@@ -13496,7 +13497,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="190" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:13" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A190" s="4">
         <v>2</v>
       </c>
@@ -13781,7 +13782,7 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="197" spans="1:22" ht="48" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:22" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A197" s="4">
         <v>2</v>
       </c>
@@ -14188,7 +14189,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="207" spans="1:22" ht="64" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:22" ht="32" x14ac:dyDescent="0.2">
       <c r="A207" s="4">
         <v>2</v>
       </c>
@@ -14305,7 +14306,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="210" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:13" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A210" s="4">
         <v>2</v>
       </c>
@@ -14738,7 +14739,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="221" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:13" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A221" s="4">
         <v>2</v>
       </c>
@@ -15105,7 +15106,7 @@
         <v>1074</v>
       </c>
     </row>
-    <row r="230" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A230" s="4">
         <v>2</v>
       </c>
@@ -17679,7 +17680,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="296" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A296" s="7">
         <v>2</v>
       </c>
@@ -18342,7 +18343,7 @@
         <v>1114</v>
       </c>
     </row>
-    <row r="313" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:13" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A313" s="7">
         <v>2</v>
       </c>
@@ -19951,7 +19952,7 @@
         <v>1147</v>
       </c>
     </row>
-    <row r="354" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A354" s="7">
         <v>2</v>
       </c>
@@ -25100,7 +25101,7 @@
         <v>1276</v>
       </c>
     </row>
-    <row r="485" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="485" spans="1:13" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A485" s="7">
         <v>3</v>
       </c>
@@ -29139,7 +29140,7 @@
         <v>1426</v>
       </c>
     </row>
-    <row r="588" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="588" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A588" s="7">
         <v>3</v>
       </c>
@@ -30272,7 +30273,7 @@
         <v>1470</v>
       </c>
     </row>
-    <row r="617" spans="1:13" ht="32" x14ac:dyDescent="0.2">
+    <row r="617" spans="1:13" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A617" s="7">
         <v>4</v>
       </c>
@@ -30959,7 +30960,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="634" spans="1:13" ht="64" x14ac:dyDescent="0.2">
+    <row r="634" spans="1:13" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A634" s="7">
         <v>4</v>
       </c>
@@ -31244,7 +31245,7 @@
         <v>1478</v>
       </c>
     </row>
-    <row r="641" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="641" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A641" s="7">
         <v>4</v>
       </c>
@@ -32552,7 +32553,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="673" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="673" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A673" s="7">
         <v>4</v>
       </c>
@@ -33674,7 +33675,7 @@
         <v>1492</v>
       </c>
     </row>
-    <row r="701" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="701" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A701" s="7">
         <v>4</v>
       </c>
@@ -34820,7 +34821,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="729" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="729" spans="1:13" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A729" s="7">
         <v>4</v>
       </c>
@@ -36093,6 +36094,13 @@
       <c r="G772" s="39"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:M759" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="SÍ"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="F46">
     <cfRule type="duplicateValues" dxfId="75" priority="76"/>
   </conditionalFormatting>
@@ -39856,6 +39864,34 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5787594d-7f52-4c24-bbc4-c61f1968f50c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0394fe40-7240-4a7e-b215-2c42bd13ce67" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="5787594d-7f52-4c24-bbc4-c61f1968f50c" xsi:nil="true"/>
+    <SharedWithUsers xmlns="0394fe40-7240-4a7e-b215-2c42bd13ce67">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007BF9F0438AAD7B4C8F3AB849F25DACE2" ma:contentTypeVersion="15" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="78dc9e79b09a45d5791aa6a49e25556e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5787594d-7f52-4c24-bbc4-c61f1968f50c" xmlns:ns3="0394fe40-7240-4a7e-b215-2c42bd13ce67" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9d38aeecf0d4424c407de8bc70dabc0" ns2:_="" ns3:_="">
     <xsd:import namespace="5787594d-7f52-4c24-bbc4-c61f1968f50c"/>
@@ -40090,35 +40126,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0CCCEFED-224C-4A22-A575-BB59C303221C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="0394fe40-7240-4a7e-b215-2c42bd13ce67"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="5787594d-7f52-4c24-bbc4-c61f1968f50c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5787594d-7f52-4c24-bbc4-c61f1968f50c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="0394fe40-7240-4a7e-b215-2c42bd13ce67" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="5787594d-7f52-4c24-bbc4-c61f1968f50c" xsi:nil="true"/>
-    <SharedWithUsers xmlns="0394fe40-7240-4a7e-b215-2c42bd13ce67">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B619118E-4560-4352-98CC-B27169FE2A24}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A7A55C-B2CE-4146-A60C-9460B5565D16}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -40135,29 +40168,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B619118E-4560-4352-98CC-B27169FE2A24}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0CCCEFED-224C-4A22-A575-BB59C303221C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="0394fe40-7240-4a7e-b215-2c42bd13ce67"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="5787594d-7f52-4c24-bbc4-c61f1968f50c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>